<commit_message>
Added Procedure Category related CS and VS and updated ServiceRequest
</commit_message>
<xml_diff>
--- a/314e-ig/output/StructureDefinition-servicerequest-314e.xlsx
+++ b/314e-ig/output/StructureDefinition-servicerequest-314e.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AO$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AO$51</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1924" uniqueCount="483">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-16T07:30:07+05:30</t>
+    <t>2026-05-16T10:04:42+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -701,11 +701,12 @@
 </t>
   </si>
   <si>
-    <t>High-level category classification for the requested service</t>
-  </si>
-  <si>
-    <t>Categorizes the requested service into a standardized
-high-level clinical service domain.</t>
+    <t>Operational procedure/service categories</t>
+  </si>
+  <si>
+    <t>Broad and optional subcategory classifications used
+for workflow, routing, analytics, and operational
+grouping of ServiceRequest resources.</t>
   </si>
   <si>
     <t>There may be multiple axis of categorization depending on the context or use case for retrieving or displaying the resource.  The level of granularity is defined by the category concepts in the value set.</t>
@@ -714,7 +715,13 @@
     <t>Used for filtering what service request are retrieved and displayed.</t>
   </si>
   <si>
-    <t>http://314e.com/fhir/ValueSet/servicerequest-category-314e</t>
+    <t>example</t>
+  </si>
+  <si>
+    <t>Classification of the requested service.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/servicerequest-category</t>
   </si>
   <si>
     <t xml:space="preserve">pattern:$this}
@@ -748,6 +755,38 @@
     <t>http://hl7.org/fhir/us/core/ValueSet/us-core-servicerequest-category</t>
   </si>
   <si>
+    <t>ServiceRequest.category:broadCategory</t>
+  </si>
+  <si>
+    <t>broadCategory</t>
+  </si>
+  <si>
+    <t>Required broad procedure/service category</t>
+  </si>
+  <si>
+    <t>Top-level operational classification of the requested
+service or procedure.</t>
+  </si>
+  <si>
+    <t>http://314e.com/fhir/ValueSet/procedure-category-broad-314e</t>
+  </si>
+  <si>
+    <t>ServiceRequest.category:subCategory</t>
+  </si>
+  <si>
+    <t>subCategory</t>
+  </si>
+  <si>
+    <t>Optional detailed subcategory</t>
+  </si>
+  <si>
+    <t>More granular operational sub-classification of the
+requested service or procedure.</t>
+  </si>
+  <si>
+    <t>http://314e.com/fhir/ValueSet/procedure-category-subcategory-314e</t>
+  </si>
+  <si>
     <t>ServiceRequest.priority</t>
   </si>
   <si>
@@ -973,9 +1012,6 @@
   </si>
   <si>
     <t>For information from the medical record intended to support the delivery of the requested services, use the `supportingInformation` element.</t>
-  </si>
-  <si>
-    <t>example</t>
   </si>
   <si>
     <t>Codified order entry details which are based on order context.</t>
@@ -1815,12 +1851,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AO49"/>
+  <dimension ref="A1:AO51"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="36.640625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="30.87890625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="11.12890625" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="12.8671875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="38.546875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.29296875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.21484375" customWidth="true" bestFit="true"/>
@@ -4035,24 +4071,26 @@
         <v>20</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>199</v>
-      </c>
-      <c r="Y19" s="2"/>
+        <v>222</v>
+      </c>
+      <c r="Y19" t="s" s="2">
+        <v>223</v>
+      </c>
       <c r="Z19" t="s" s="2">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AB19" t="s" s="2">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="AC19" s="2"/>
       <c r="AD19" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE19" t="s" s="2">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="AF19" t="s" s="2">
         <v>216</v>
@@ -4073,10 +4111,10 @@
         <v>20</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="AM19" t="s" s="2">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="AN19" t="s" s="2">
         <v>215</v>
@@ -4087,13 +4125,13 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B20" t="s" s="2">
         <v>216</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D20" t="s" s="2">
         <v>20</v>
@@ -4118,10 +4156,10 @@
         <v>217</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="N20" t="s" s="2">
         <v>220</v>
@@ -4155,10 +4193,10 @@
         <v>199</v>
       </c>
       <c r="Y20" t="s" s="2">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="Z20" t="s" s="2">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>20</v>
@@ -4194,10 +4232,10 @@
         <v>20</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="AN20" t="s" s="2">
         <v>215</v>
@@ -4206,26 +4244,28 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" hidden="true">
+    <row r="21">
       <c r="A21" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>233</v>
-      </c>
-      <c r="C21" s="2"/>
+        <v>216</v>
+      </c>
+      <c r="C21" t="s" s="2">
+        <v>236</v>
+      </c>
       <c r="D21" t="s" s="2">
         <v>20</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G21" t="s" s="2">
         <v>90</v>
       </c>
       <c r="H21" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="I21" t="s" s="2">
         <v>20</v>
@@ -4234,22 +4274,24 @@
         <v>91</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>110</v>
+        <v>217</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>235</v>
-      </c>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
+        <v>238</v>
+      </c>
+      <c r="N21" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="O21" t="s" s="2">
+        <v>221</v>
+      </c>
       <c r="P21" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="Q21" t="s" s="2">
-        <v>236</v>
-      </c>
+      <c r="Q21" s="2"/>
       <c r="R21" t="s" s="2">
         <v>20</v>
       </c>
@@ -4271,11 +4313,9 @@
       <c r="X21" t="s" s="2">
         <v>199</v>
       </c>
-      <c r="Y21" t="s" s="2">
-        <v>237</v>
-      </c>
+      <c r="Y21" s="2"/>
       <c r="Z21" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>20</v>
@@ -4293,13 +4333,13 @@
         <v>20</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>233</v>
+        <v>216</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH21" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI21" t="s" s="2">
         <v>20</v>
@@ -4308,29 +4348,31 @@
         <v>102</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>239</v>
+        <v>20</v>
       </c>
       <c r="AL21" t="s" s="2">
+        <v>227</v>
+      </c>
+      <c r="AM21" t="s" s="2">
+        <v>228</v>
+      </c>
+      <c r="AN21" t="s" s="2">
+        <v>215</v>
+      </c>
+      <c r="AO21" t="s" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="AM21" t="s" s="2">
+      <c r="B22" t="s" s="2">
+        <v>216</v>
+      </c>
+      <c r="C22" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="AN21" t="s" s="2">
-        <v>242</v>
-      </c>
-      <c r="AO21" t="s" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" hidden="true">
-      <c r="A22" t="s" s="2">
-        <v>243</v>
-      </c>
-      <c r="B22" t="s" s="2">
-        <v>243</v>
-      </c>
-      <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
         <v>20</v>
       </c>
@@ -4342,62 +4384,58 @@
         <v>90</v>
       </c>
       <c r="H22" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="I22" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="J22" t="s" s="2">
         <v>91</v>
       </c>
       <c r="K22" t="s" s="2">
+        <v>217</v>
+      </c>
+      <c r="L22" t="s" s="2">
+        <v>242</v>
+      </c>
+      <c r="M22" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="N22" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="O22" t="s" s="2">
+        <v>221</v>
+      </c>
+      <c r="P22" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Q22" s="2"/>
+      <c r="R22" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="S22" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="T22" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="U22" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V22" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W22" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X22" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="Y22" s="2"/>
+      <c r="Z22" t="s" s="2">
         <v>244</v>
       </c>
-      <c r="L22" t="s" s="2">
-        <v>245</v>
-      </c>
-      <c r="M22" t="s" s="2">
-        <v>246</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="O22" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="P22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Q22" t="s" s="2">
-        <v>249</v>
-      </c>
-      <c r="R22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="S22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="T22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="U22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="V22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="W22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="X22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Y22" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Z22" t="s" s="2">
-        <v>20</v>
-      </c>
       <c r="AA22" t="s" s="2">
         <v>20</v>
       </c>
@@ -4414,13 +4452,13 @@
         <v>20</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>243</v>
+        <v>216</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>20</v>
@@ -4429,41 +4467,41 @@
         <v>102</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>250</v>
+        <v>20</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>20</v>
+        <v>227</v>
       </c>
       <c r="AM22" t="s" s="2">
-        <v>251</v>
+        <v>228</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>20</v>
+        <v>215</v>
       </c>
       <c r="AO22" t="s" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>253</v>
+        <v>20</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G23" t="s" s="2">
         <v>90</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>20</v>
@@ -4472,22 +4510,22 @@
         <v>91</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>217</v>
+        <v>110</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>255</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>256</v>
-      </c>
+        <v>247</v>
+      </c>
+      <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="Q23" s="2"/>
+      <c r="Q23" t="s" s="2">
+        <v>248</v>
+      </c>
       <c r="R23" t="s" s="2">
         <v>20</v>
       </c>
@@ -4507,11 +4545,13 @@
         <v>20</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>257</v>
-      </c>
-      <c r="Y23" s="2"/>
+        <v>199</v>
+      </c>
+      <c r="Y23" t="s" s="2">
+        <v>249</v>
+      </c>
       <c r="Z23" t="s" s="2">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>20</v>
@@ -4529,7 +4569,7 @@
         <v>20</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>80</v>
@@ -4538,33 +4578,33 @@
         <v>90</v>
       </c>
       <c r="AI23" t="s" s="2">
-        <v>259</v>
+        <v>20</v>
       </c>
       <c r="AJ23" t="s" s="2">
         <v>102</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>264</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4581,26 +4621,32 @@
         <v>20</v>
       </c>
       <c r="I24" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>268</v>
-      </c>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
+        <v>258</v>
+      </c>
+      <c r="N24" t="s" s="2">
+        <v>259</v>
+      </c>
+      <c r="O24" t="s" s="2">
+        <v>260</v>
+      </c>
       <c r="P24" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="Q24" s="2"/>
+      <c r="Q24" t="s" s="2">
+        <v>261</v>
+      </c>
       <c r="R24" t="s" s="2">
         <v>20</v>
       </c>
@@ -4644,7 +4690,7 @@
         <v>20</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>80</v>
@@ -4656,16 +4702,16 @@
         <v>20</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>20</v>
+        <v>102</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>20</v>
+        <v>262</v>
       </c>
       <c r="AL24" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="AN24" t="s" s="2">
         <v>20</v>
@@ -4674,44 +4720,44 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" hidden="true">
+    <row r="25">
       <c r="A25" t="s" s="2">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>135</v>
+        <v>265</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H25" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="I25" t="s" s="2">
         <v>20</v>
       </c>
       <c r="J25" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>136</v>
+        <v>217</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>137</v>
+        <v>266</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>139</v>
+        <v>268</v>
       </c>
       <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
@@ -4737,70 +4783,66 @@
         <v>20</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Y25" t="s" s="2">
-        <v>20</v>
-      </c>
+        <v>269</v>
+      </c>
+      <c r="Y25" s="2"/>
       <c r="Z25" t="s" s="2">
-        <v>20</v>
+        <v>270</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AB25" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC25" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD25" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE25" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF25" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="AG25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH25" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI25" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="AJ25" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK25" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="AL25" t="s" s="2">
         <v>273</v>
       </c>
-      <c r="AC25" t="s" s="2">
+      <c r="AM25" t="s" s="2">
         <v>274</v>
       </c>
-      <c r="AD25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AE25" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="AF25" t="s" s="2">
+      <c r="AN25" t="s" s="2">
         <v>275</v>
       </c>
-      <c r="AG25" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH25" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AJ25" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="AK25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AL25" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AM25" t="s" s="2">
-        <v>270</v>
-      </c>
-      <c r="AN25" t="s" s="2">
-        <v>20</v>
-      </c>
       <c r="AO25" t="s" s="2">
-        <v>20</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>271</v>
-      </c>
-      <c r="C26" t="s" s="2">
         <v>277</v>
       </c>
+      <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
         <v>20</v>
       </c>
@@ -4829,9 +4871,7 @@
       <c r="M26" t="s" s="2">
         <v>280</v>
       </c>
-      <c r="N26" t="s" s="2">
-        <v>281</v>
-      </c>
+      <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
         <v>20</v>
@@ -4880,28 +4920,28 @@
         <v>20</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH26" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI26" t="s" s="2">
-        <v>259</v>
+        <v>20</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>141</v>
+        <v>20</v>
       </c>
       <c r="AK26" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL26" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM26" t="s" s="2">
         <v>282</v>
-      </c>
-      <c r="AM26" t="s" s="2">
-        <v>283</v>
       </c>
       <c r="AN26" t="s" s="2">
         <v>20</v>
@@ -4912,14 +4952,14 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>20</v>
+        <v>135</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
@@ -4935,23 +4975,21 @@
         <v>20</v>
       </c>
       <c r="J27" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>285</v>
+        <v>136</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>286</v>
+        <v>137</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="O27" t="s" s="2">
-        <v>289</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
         <v>20</v>
       </c>
@@ -4987,19 +5025,19 @@
         <v>20</v>
       </c>
       <c r="AB27" t="s" s="2">
-        <v>20</v>
+        <v>285</v>
       </c>
       <c r="AC27" t="s" s="2">
-        <v>20</v>
+        <v>286</v>
       </c>
       <c r="AD27" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE27" t="s" s="2">
-        <v>20</v>
+        <v>226</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>80</v>
@@ -5011,16 +5049,16 @@
         <v>20</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>291</v>
+        <v>20</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="AN27" t="s" s="2">
         <v>20</v>
@@ -5031,12 +5069,14 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>293</v>
-      </c>
-      <c r="C28" s="2"/>
+        <v>283</v>
+      </c>
+      <c r="C28" t="s" s="2">
+        <v>289</v>
+      </c>
       <c r="D28" t="s" s="2">
         <v>20</v>
       </c>
@@ -5054,23 +5094,21 @@
         <v>20</v>
       </c>
       <c r="J28" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>266</v>
+        <v>290</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>296</v>
-      </c>
-      <c r="O28" t="s" s="2">
-        <v>297</v>
-      </c>
+        <v>293</v>
+      </c>
+      <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>20</v>
       </c>
@@ -5118,28 +5156,28 @@
         <v>20</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI28" t="s" s="2">
-        <v>20</v>
+        <v>271</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="AK28" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="AN28" t="s" s="2">
         <v>20</v>
@@ -5150,14 +5188,14 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>302</v>
+        <v>20</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -5176,18 +5214,20 @@
         <v>91</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>217</v>
+        <v>297</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="O29" s="2"/>
+        <v>300</v>
+      </c>
+      <c r="O29" t="s" s="2">
+        <v>301</v>
+      </c>
       <c r="P29" t="s" s="2">
         <v>20</v>
       </c>
@@ -5211,13 +5251,13 @@
         <v>20</v>
       </c>
       <c r="X29" t="s" s="2">
-        <v>306</v>
+        <v>20</v>
       </c>
       <c r="Y29" t="s" s="2">
-        <v>307</v>
+        <v>20</v>
       </c>
       <c r="Z29" t="s" s="2">
-        <v>308</v>
+        <v>20</v>
       </c>
       <c r="AA29" t="s" s="2">
         <v>20</v>
@@ -5235,7 +5275,7 @@
         <v>20</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>80</v>
@@ -5244,7 +5284,7 @@
         <v>81</v>
       </c>
       <c r="AI29" t="s" s="2">
-        <v>309</v>
+        <v>20</v>
       </c>
       <c r="AJ29" t="s" s="2">
         <v>102</v>
@@ -5253,24 +5293,24 @@
         <v>20</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>262</v>
+        <v>304</v>
       </c>
       <c r="AN29" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AO29" t="s" s="2">
-        <v>264</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5293,17 +5333,19 @@
         <v>91</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>312</v>
+        <v>278</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>314</v>
-      </c>
-      <c r="N30" s="2"/>
+        <v>307</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>308</v>
+      </c>
       <c r="O30" t="s" s="2">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>20</v>
@@ -5352,7 +5394,7 @@
         <v>20</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>80</v>
@@ -5370,10 +5412,10 @@
         <v>20</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="AN30" t="s" s="2">
         <v>20</v>
@@ -5382,26 +5424,26 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>20</v>
+        <v>314</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>20</v>
@@ -5410,15 +5452,17 @@
         <v>91</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>318</v>
+        <v>217</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>320</v>
-      </c>
-      <c r="N31" s="2"/>
+        <v>316</v>
+      </c>
+      <c r="N31" t="s" s="2">
+        <v>317</v>
+      </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>20</v>
@@ -5443,13 +5487,13 @@
         <v>20</v>
       </c>
       <c r="X31" t="s" s="2">
-        <v>20</v>
+        <v>222</v>
       </c>
       <c r="Y31" t="s" s="2">
-        <v>20</v>
+        <v>318</v>
       </c>
       <c r="Z31" t="s" s="2">
-        <v>20</v>
+        <v>319</v>
       </c>
       <c r="AA31" t="s" s="2">
         <v>20</v>
@@ -5467,46 +5511,46 @@
         <v>20</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="AG31" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AH31" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI31" t="s" s="2">
-        <v>20</v>
+        <v>320</v>
       </c>
       <c r="AJ31" t="s" s="2">
         <v>102</v>
       </c>
       <c r="AK31" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AL31" t="s" s="2">
         <v>321</v>
       </c>
-      <c r="AL31" t="s" s="2">
+      <c r="AM31" t="s" s="2">
+        <v>274</v>
+      </c>
+      <c r="AN31" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AO31" t="s" s="2">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="32" hidden="true">
+      <c r="A32" t="s" s="2">
         <v>322</v>
       </c>
-      <c r="AM31" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="AN31" t="s" s="2">
-        <v>324</v>
-      </c>
-      <c r="AO31" t="s" s="2">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s" s="2">
-        <v>326</v>
-      </c>
       <c r="B32" t="s" s="2">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>327</v>
+        <v>20</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
@@ -5516,7 +5560,7 @@
         <v>90</v>
       </c>
       <c r="H32" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="I32" t="s" s="2">
         <v>20</v>
@@ -5525,16 +5569,18 @@
         <v>91</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
+      <c r="O32" t="s" s="2">
+        <v>326</v>
+      </c>
       <c r="P32" t="s" s="2">
         <v>20</v>
       </c>
@@ -5582,7 +5628,7 @@
         <v>20</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>80</v>
@@ -5597,35 +5643,35 @@
         <v>102</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>331</v>
+        <v>20</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>332</v>
+        <v>321</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>334</v>
+        <v>20</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>335</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>337</v>
+        <v>20</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G33" t="s" s="2">
         <v>90</v>
@@ -5640,13 +5686,13 @@
         <v>91</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>338</v>
+        <v>329</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -5697,10 +5743,10 @@
         <v>20</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="AG33" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AH33" t="s" s="2">
         <v>90</v>
@@ -5712,31 +5758,31 @@
         <v>102</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>345</v>
+        <v>336</v>
       </c>
     </row>
-    <row r="34" hidden="true">
+    <row r="34">
       <c r="A34" t="s" s="2">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>20</v>
+        <v>338</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -5746,7 +5792,7 @@
         <v>90</v>
       </c>
       <c r="H34" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="I34" t="s" s="2">
         <v>20</v>
@@ -5755,13 +5801,13 @@
         <v>91</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5788,13 +5834,13 @@
         <v>20</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>306</v>
+        <v>20</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>350</v>
+        <v>20</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>351</v>
+        <v>20</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>20</v>
@@ -5812,7 +5858,7 @@
         <v>20</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>80</v>
@@ -5827,31 +5873,31 @@
         <v>102</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>20</v>
+        <v>342</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>20</v>
+        <v>343</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>20</v>
+        <v>345</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>353</v>
+        <v>346</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
@@ -5870,13 +5916,13 @@
         <v>91</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -5927,7 +5973,7 @@
         <v>20</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>80</v>
@@ -5942,31 +5988,31 @@
         <v>102</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>363</v>
+        <v>356</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>365</v>
+        <v>20</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
@@ -5976,7 +6022,7 @@
         <v>90</v>
       </c>
       <c r="H36" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="I36" t="s" s="2">
         <v>20</v>
@@ -5985,17 +6031,15 @@
         <v>91</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>368</v>
-      </c>
-      <c r="N36" t="s" s="2">
-        <v>369</v>
-      </c>
+        <v>360</v>
+      </c>
+      <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>20</v>
@@ -6020,13 +6064,13 @@
         <v>20</v>
       </c>
       <c r="X36" t="s" s="2">
-        <v>20</v>
+        <v>222</v>
       </c>
       <c r="Y36" t="s" s="2">
-        <v>20</v>
+        <v>361</v>
       </c>
       <c r="Z36" t="s" s="2">
-        <v>20</v>
+        <v>362</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>20</v>
@@ -6044,7 +6088,7 @@
         <v>20</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>80</v>
@@ -6059,31 +6103,31 @@
         <v>102</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>370</v>
+        <v>20</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>371</v>
+        <v>20</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>373</v>
+        <v>20</v>
       </c>
       <c r="AO36" t="s" s="2">
-        <v>374</v>
+        <v>364</v>
       </c>
     </row>
-    <row r="37" hidden="true">
+    <row r="37">
       <c r="A37" t="s" s="2">
-        <v>375</v>
+        <v>365</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>375</v>
+        <v>365</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>376</v>
+        <v>366</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -6093,7 +6137,7 @@
         <v>90</v>
       </c>
       <c r="H37" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="I37" t="s" s="2">
         <v>20</v>
@@ -6102,17 +6146,15 @@
         <v>91</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>217</v>
+        <v>367</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>378</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>379</v>
-      </c>
+        <v>369</v>
+      </c>
+      <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>20</v>
@@ -6137,13 +6179,13 @@
         <v>20</v>
       </c>
       <c r="X37" t="s" s="2">
-        <v>306</v>
+        <v>20</v>
       </c>
       <c r="Y37" t="s" s="2">
-        <v>380</v>
+        <v>20</v>
       </c>
       <c r="Z37" t="s" s="2">
-        <v>381</v>
+        <v>20</v>
       </c>
       <c r="AA37" t="s" s="2">
         <v>20</v>
@@ -6161,7 +6203,7 @@
         <v>20</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>375</v>
+        <v>365</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>80</v>
@@ -6176,41 +6218,41 @@
         <v>102</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>382</v>
+        <v>370</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>383</v>
+        <v>371</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>385</v>
+        <v>373</v>
       </c>
       <c r="AO37" t="s" s="2">
-        <v>20</v>
+        <v>374</v>
       </c>
     </row>
-    <row r="38" hidden="true">
+    <row r="38">
       <c r="A38" t="s" s="2">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>20</v>
@@ -6219,16 +6261,16 @@
         <v>91</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>391</v>
+        <v>380</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -6278,13 +6320,13 @@
         <v>20</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>20</v>
@@ -6293,38 +6335,38 @@
         <v>102</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>394</v>
+        <v>383</v>
       </c>
       <c r="AN38" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="AO38" t="s" s="2">
         <v>385</v>
-      </c>
-      <c r="AO38" t="s" s="2">
-        <v>20</v>
       </c>
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
-        <v>20</v>
+        <v>387</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>20</v>
@@ -6339,12 +6381,14 @@
         <v>217</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>397</v>
-      </c>
-      <c r="N39" s="2"/>
+        <v>389</v>
+      </c>
+      <c r="N39" t="s" s="2">
+        <v>390</v>
+      </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>20</v>
@@ -6369,13 +6413,13 @@
         <v>20</v>
       </c>
       <c r="X39" t="s" s="2">
-        <v>306</v>
+        <v>222</v>
       </c>
       <c r="Y39" t="s" s="2">
-        <v>398</v>
+        <v>391</v>
       </c>
       <c r="Z39" t="s" s="2">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>20</v>
@@ -6393,13 +6437,13 @@
         <v>20</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="AI39" t="s" s="2">
         <v>20</v>
@@ -6408,16 +6452,16 @@
         <v>102</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>20</v>
+        <v>393</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>20</v>
+        <v>394</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="AN39" t="s" s="2">
-        <v>385</v>
+        <v>396</v>
       </c>
       <c r="AO39" t="s" s="2">
         <v>20</v>
@@ -6425,14 +6469,14 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>20</v>
+        <v>398</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
@@ -6451,15 +6495,17 @@
         <v>91</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>399</v>
+      </c>
+      <c r="L40" t="s" s="2">
+        <v>400</v>
+      </c>
+      <c r="M40" t="s" s="2">
+        <v>401</v>
+      </c>
+      <c r="N40" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="L40" t="s" s="2">
-        <v>396</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>403</v>
-      </c>
-      <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>20</v>
@@ -6508,7 +6554,7 @@
         <v>20</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>80</v>
@@ -6523,16 +6569,16 @@
         <v>102</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>20</v>
+        <v>403</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>20</v>
+        <v>404</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>385</v>
+        <v>396</v>
       </c>
       <c r="AO40" t="s" s="2">
         <v>20</v>
@@ -6540,10 +6586,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6569,14 +6615,12 @@
         <v>217</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>407</v>
-      </c>
-      <c r="N41" t="s" s="2">
         <v>408</v>
       </c>
+      <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>20</v>
@@ -6601,11 +6645,13 @@
         <v>20</v>
       </c>
       <c r="X41" t="s" s="2">
-        <v>257</v>
-      </c>
-      <c r="Y41" s="2"/>
+        <v>222</v>
+      </c>
+      <c r="Y41" t="s" s="2">
+        <v>409</v>
+      </c>
       <c r="Z41" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>20</v>
@@ -6623,7 +6669,7 @@
         <v>20</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>80</v>
@@ -6638,16 +6684,16 @@
         <v>102</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>410</v>
+        <v>20</v>
       </c>
       <c r="AL41" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AM41" t="s" s="2">
         <v>411</v>
       </c>
-      <c r="AM41" t="s" s="2">
-        <v>412</v>
-      </c>
       <c r="AN41" t="s" s="2">
-        <v>413</v>
+        <v>396</v>
       </c>
       <c r="AO41" t="s" s="2">
         <v>20</v>
@@ -6655,10 +6701,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6681,17 +6727,15 @@
         <v>91</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>416</v>
+        <v>407</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>417</v>
-      </c>
-      <c r="N42" t="s" s="2">
-        <v>418</v>
-      </c>
+        <v>414</v>
+      </c>
+      <c r="N42" s="2"/>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
         <v>20</v>
@@ -6740,7 +6784,7 @@
         <v>20</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>80</v>
@@ -6755,16 +6799,16 @@
         <v>102</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>419</v>
+        <v>20</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>420</v>
+        <v>20</v>
       </c>
       <c r="AM42" t="s" s="2">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>413</v>
+        <v>396</v>
       </c>
       <c r="AO42" t="s" s="2">
         <v>20</v>
@@ -6772,10 +6816,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6795,18 +6839,20 @@
         <v>20</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>423</v>
+        <v>217</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>425</v>
-      </c>
-      <c r="N43" s="2"/>
+        <v>418</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>419</v>
+      </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>20</v>
@@ -6831,13 +6877,11 @@
         <v>20</v>
       </c>
       <c r="X43" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Y43" t="s" s="2">
-        <v>20</v>
-      </c>
+        <v>269</v>
+      </c>
+      <c r="Y43" s="2"/>
       <c r="Z43" t="s" s="2">
-        <v>20</v>
+        <v>420</v>
       </c>
       <c r="AA43" t="s" s="2">
         <v>20</v>
@@ -6855,7 +6899,7 @@
         <v>20</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>80</v>
@@ -6870,16 +6914,16 @@
         <v>102</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="AM43" t="s" s="2">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>20</v>
+        <v>424</v>
       </c>
       <c r="AO43" t="s" s="2">
         <v>20</v>
@@ -6887,14 +6931,14 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>430</v>
+        <v>20</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -6910,19 +6954,19 @@
         <v>20</v>
       </c>
       <c r="J44" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="N44" t="s" s="2">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
@@ -6972,7 +7016,7 @@
         <v>20</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>80</v>
@@ -6987,16 +7031,16 @@
         <v>102</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="AM44" t="s" s="2">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="AN44" t="s" s="2">
-        <v>20</v>
+        <v>424</v>
       </c>
       <c r="AO44" t="s" s="2">
         <v>20</v>
@@ -7004,10 +7048,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -7027,20 +7071,18 @@
         <v>20</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>441</v>
-      </c>
-      <c r="N45" t="s" s="2">
-        <v>442</v>
-      </c>
+        <v>436</v>
+      </c>
+      <c r="N45" s="2"/>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>20</v>
@@ -7089,7 +7131,7 @@
         <v>20</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>80</v>
@@ -7104,13 +7146,13 @@
         <v>102</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>20</v>
+        <v>437</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="AN45" t="s" s="2">
         <v>20</v>
@@ -7121,14 +7163,14 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
@@ -7144,23 +7186,21 @@
         <v>20</v>
       </c>
       <c r="J46" t="s" s="2">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>217</v>
+        <v>442</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>449</v>
-      </c>
-      <c r="O46" t="s" s="2">
-        <v>450</v>
-      </c>
+        <v>445</v>
+      </c>
+      <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>20</v>
       </c>
@@ -7184,13 +7224,13 @@
         <v>20</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>306</v>
+        <v>20</v>
       </c>
       <c r="Y46" t="s" s="2">
-        <v>451</v>
+        <v>20</v>
       </c>
       <c r="Z46" t="s" s="2">
-        <v>452</v>
+        <v>20</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>20</v>
@@ -7208,7 +7248,7 @@
         <v>20</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>80</v>
@@ -7223,27 +7263,27 @@
         <v>102</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>20</v>
+        <v>446</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="AN46" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>454</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7263,18 +7303,20 @@
         <v>20</v>
       </c>
       <c r="J47" t="s" s="2">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>51</v>
+        <v>451</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>457</v>
-      </c>
-      <c r="N47" s="2"/>
+        <v>452</v>
+      </c>
+      <c r="N47" t="s" s="2">
+        <v>453</v>
+      </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
         <v>20</v>
@@ -7323,7 +7365,7 @@
         <v>20</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>80</v>
@@ -7338,38 +7380,38 @@
         <v>102</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>458</v>
+        <v>20</v>
       </c>
       <c r="AL47" t="s" s="2">
-        <v>310</v>
+        <v>454</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="AN47" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AO47" t="s" s="2">
-        <v>460</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
-        <v>20</v>
+        <v>457</v>
       </c>
       <c r="E48" s="2"/>
       <c r="F48" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>20</v>
@@ -7381,16 +7423,20 @@
         <v>91</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>266</v>
+        <v>217</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>463</v>
-      </c>
-      <c r="N48" s="2"/>
-      <c r="O48" s="2"/>
+        <v>459</v>
+      </c>
+      <c r="N48" t="s" s="2">
+        <v>460</v>
+      </c>
+      <c r="O48" t="s" s="2">
+        <v>461</v>
+      </c>
       <c r="P48" t="s" s="2">
         <v>20</v>
       </c>
@@ -7414,13 +7460,13 @@
         <v>20</v>
       </c>
       <c r="X48" t="s" s="2">
-        <v>20</v>
+        <v>222</v>
       </c>
       <c r="Y48" t="s" s="2">
-        <v>20</v>
+        <v>462</v>
       </c>
       <c r="Z48" t="s" s="2">
-        <v>20</v>
+        <v>463</v>
       </c>
       <c r="AA48" t="s" s="2">
         <v>20</v>
@@ -7438,13 +7484,13 @@
         <v>20</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AI48" t="s" s="2">
         <v>20</v>
@@ -7456,7 +7502,7 @@
         <v>20</v>
       </c>
       <c r="AL48" t="s" s="2">
-        <v>310</v>
+        <v>454</v>
       </c>
       <c r="AM48" t="s" s="2">
         <v>464</v>
@@ -7465,15 +7511,15 @@
         <v>20</v>
       </c>
       <c r="AO48" t="s" s="2">
-        <v>20</v>
+        <v>465</v>
       </c>
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7496,17 +7542,15 @@
         <v>20</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>467</v>
+        <v>51</v>
       </c>
       <c r="M49" t="s" s="2">
         <v>468</v>
       </c>
-      <c r="N49" t="s" s="2">
-        <v>469</v>
-      </c>
+      <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
         <v>20</v>
@@ -7555,7 +7599,7 @@
         <v>20</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>80</v>
@@ -7570,23 +7614,255 @@
         <v>102</v>
       </c>
       <c r="AK49" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="AL49" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="AM49" t="s" s="2">
         <v>470</v>
       </c>
-      <c r="AL49" t="s" s="2">
+      <c r="AN49" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AO49" t="s" s="2">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="50" hidden="true">
+      <c r="A50" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="B50" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="E50" s="2"/>
+      <c r="F50" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G50" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="I50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="J50" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="K50" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="L50" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="M50" t="s" s="2">
+        <v>474</v>
+      </c>
+      <c r="N50" s="2"/>
+      <c r="O50" s="2"/>
+      <c r="P50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Q50" s="2"/>
+      <c r="R50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="S50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="T50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="U50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Y50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Z50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AA50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF50" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="AG50" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH50" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AJ50" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AL50" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="AM50" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="AN50" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AO50" t="s" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51" hidden="true">
+      <c r="A51" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="B51" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="C51" s="2"/>
+      <c r="D51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="E51" s="2"/>
+      <c r="F51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="H51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="I51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="J51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="K51" t="s" s="2">
+        <v>477</v>
+      </c>
+      <c r="L51" t="s" s="2">
+        <v>478</v>
+      </c>
+      <c r="M51" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="N51" t="s" s="2">
+        <v>480</v>
+      </c>
+      <c r="O51" s="2"/>
+      <c r="P51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Q51" s="2"/>
+      <c r="R51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="S51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="T51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="U51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="V51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="W51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="X51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Y51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Z51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AA51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AB51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AC51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AD51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AE51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AF51" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="AG51" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AH51" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AI51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AJ51" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="AK51" t="s" s="2">
+        <v>481</v>
+      </c>
+      <c r="AL51" t="s" s="2">
         <v>133</v>
       </c>
-      <c r="AM49" t="s" s="2">
-        <v>471</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AO49" t="s" s="2">
+      <c r="AM51" t="s" s="2">
+        <v>482</v>
+      </c>
+      <c r="AN51" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AO51" t="s" s="2">
         <v>20</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AO49">
+  <autoFilter ref="A1:AO51">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -7596,7 +7872,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI48">
+  <conditionalFormatting sqref="A2:AI50">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>